<commit_message>
2nd frontend dev changes
</commit_message>
<xml_diff>
--- a/wiki/development-plan/notion-finance-development-plan.xlsx
+++ b/wiki/development-plan/notion-finance-development-plan.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R37035b11e9c74b2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frontend-dev-plan" sheetId="2" r:id="Reddf22f3d76f4aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backend-dev-plan" sheetId="3" r:id="R79579aa231e64cc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="integration-dev-plan" sheetId="4" r:id="Rb8dd331d8daa4714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="testing-dev-plan" sheetId="5" r:id="Rec0fd0611279410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf46e0e4d0d894d24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frontend-dev-plan" sheetId="2" r:id="R285227dcec9a444b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backend-dev-plan" sheetId="3" r:id="Rf1327151e5244157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="integration-dev-plan" sheetId="4" r:id="R10b6a63a6bef4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="testing-dev-plan" sheetId="5" r:id="Re060937ae05c4d3d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -706,7 +706,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="17" t="str">
-        <x:v>Updated 2026-07-03. Frontend implementation now includes prototype-aligned dashboard list, modal-first create/edit flows, Monitoring category views, and the Next.js workspace foundation while Notion remains the source of truth.</x:v>
+        <x:v>Updated 2026-07-04. Backend plan is aligned to the current read-only Accounts, Income Categories, and Expense Categories design while frontend implementation remains in progress and Notion remains the source of truth.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -1000,10 +1000,8 @@
           <x:t xml:space="preserve">Recommended next move</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Document duplicated Notion access details, confirm compact/detail fields, and verify Alkansya backing view during implementation discovery.</x:t>
-        </x:is>
+      <x:c r="E16" s="30" t="str">
+        <x:v>Document duplicated Notion access details, confirm compact/detail fields, and confirm live relation/category mappings during backend implementation discovery.</x:v>
       </x:c>
       <x:c r="F16" s="30" t="n"/>
       <x:c r="G16" s="30" t="n"/>
@@ -1093,25 +1091,17 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="29" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Account Delete</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deleting an account marks it inactive. It does not delete the Notion record.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Resolved</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Product, Backend</x:t>
-        </x:is>
+      <x:c r="A23" s="29" t="str">
+        <x:v>Reference Data Maintenance</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>Accounts, income categories, and expense categories are maintained in Notion only; the app exposes reads only.</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>Resolved</x:v>
+      </x:c>
+      <x:c r="D23" s="30" t="str">
+        <x:v>Product, Backend</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
@@ -2479,1471 +2469,917 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="15" customHeight="1">
-      <x:c r="A4" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ID</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Priority</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Epic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Work Item</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Owner Role</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Dependencies</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Acceptance Criteria</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Status</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Blocked / Decision Needed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Verification / Evidence</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Source Docs</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Notes</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N4" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Last Updated</x:t>
-        </x:is>
+      <x:c r="A4" s="1" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>Phase</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="str">
+        <x:v>Work Item</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="str">
+        <x:v>Owner Role</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="str">
+        <x:v>Dependencies</x:v>
+      </x:c>
+      <x:c r="H4" s="2" t="str">
+        <x:v>Acceptance Criteria</x:v>
+      </x:c>
+      <x:c r="I4" s="2" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="J4" s="2" t="str">
+        <x:v>Blocked / Decision Needed</x:v>
+      </x:c>
+      <x:c r="K4" s="2" t="str">
+        <x:v>Verification / Evidence</x:v>
+      </x:c>
+      <x:c r="L4" s="2" t="str">
+        <x:v>Source Docs</x:v>
+      </x:c>
+      <x:c r="M4" s="2" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+      <x:c r="N4" s="3" t="str">
+        <x:v>Last Updated</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="25.5" customHeight="1">
-      <x:c r="A5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-001</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Foundation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Service Scaffold</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Scaffold NestJS service in service/</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implementation approval</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NestJS service exists under service/ with health endpoint, scripts, lint/typecheck/test placeholders, and environment loading baseline</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I5" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current phase says no application source code yet</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build/lint/typecheck commands pass once tooling exists</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/project-structure/project-structure.md; wiki/tdd/tdd.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Do this only after planning approval</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N5" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A5" s="4" t="str">
+        <x:v>BE-001</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>Foundation</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>Service Scaffold</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>Scaffold NestJS service in service/</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="str">
+        <x:v>Implementation approval</x:v>
+      </x:c>
+      <x:c r="H5" s="4" t="str">
+        <x:v>NestJS service exists under service/ with health endpoint, scripts, lint/typecheck/test placeholders, and environment loading baseline</x:v>
+      </x:c>
+      <x:c r="I5" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J5" s="4" t="str">
+        <x:v>Pending explicit backend implementation request</x:v>
+      </x:c>
+      <x:c r="K5" s="4" t="str">
+        <x:v>Build/lint/typecheck commands pass once tooling exists</x:v>
+      </x:c>
+      <x:c r="L5" s="4" t="str">
+        <x:v>wiki/project-structure/project-structure.md; wiki/tdd/tdd.md</x:v>
+      </x:c>
+      <x:c r="M5" s="4" t="str">
+        <x:v>Do this only after backend implementation approval.</x:v>
+      </x:c>
+      <x:c r="N5" s="4" t="str">
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38.25" customHeight="1">
-      <x:c r="A6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-002</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Foundation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Configuration</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implement server-side configuration and secret loading</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer, Security Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-001</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Notion token, database IDs, metadata store settings, and environment-specific options are read server-side only and validated on startup</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I6" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J6" s="30" t="n"/>
-      <x:c r="K6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit tests and secret scan</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/tdd/tdd.md; wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Do not expose token or server-only env values to application/</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N6" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A6" s="30" t="str">
+        <x:v>BE-002</x:v>
+      </x:c>
+      <x:c r="B6" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="30" t="str">
+        <x:v>Foundation</x:v>
+      </x:c>
+      <x:c r="D6" s="30" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="E6" s="30" t="str">
+        <x:v>Implement server-side configuration and secret loading</x:v>
+      </x:c>
+      <x:c r="F6" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer, Security Engineer</x:v>
+      </x:c>
+      <x:c r="G6" s="30" t="str">
+        <x:v>BE-001</x:v>
+      </x:c>
+      <x:c r="H6" s="30" t="str">
+        <x:v>Notion token, database IDs, metadata store settings, and environment-specific options are read server-side only and validated on startup</x:v>
+      </x:c>
+      <x:c r="I6" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J6" s="30"/>
+      <x:c r="K6" s="30" t="str">
+        <x:v>Unit tests and secret scan</x:v>
+      </x:c>
+      <x:c r="L6" s="30" t="str">
+        <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
+      </x:c>
+      <x:c r="M6" s="30" t="str">
+        <x:v>Do not expose token or server-only env values to application/</x:v>
+      </x:c>
+      <x:c r="N6" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25.5" customHeight="1">
-      <x:c r="A7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-003</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planning</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Authentication</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Decide and implement MVP auth/session model</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Security Engineer, Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP auth decision</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Email sign-in and Google sign-in are implemented; write endpoints and sync commit are protected</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I7" s="25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J7" s="30" t="str"/>
-      <x:c r="K7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Auth tests for email sign-in, Google sign-in, session/me, logout, and protected routes</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/product-specification/product-specification.md; wiki/api/api-specification.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Decision: auth is required for multi-user use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N7" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A7" s="30" t="str">
+        <x:v>BE-003</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>Planning</x:v>
+      </x:c>
+      <x:c r="D7" s="30" t="str">
+        <x:v>Authentication</x:v>
+      </x:c>
+      <x:c r="E7" s="30" t="str">
+        <x:v>Decide and implement MVP auth/session model</x:v>
+      </x:c>
+      <x:c r="F7" s="30" t="str">
+        <x:v>Security Engineer, Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G7" s="30" t="str">
+        <x:v>MVP auth decision</x:v>
+      </x:c>
+      <x:c r="H7" s="30" t="str">
+        <x:v>Email sign-in and Google sign-in are implemented; write endpoints and sync commit are protected</x:v>
+      </x:c>
+      <x:c r="I7" s="25" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J7" s="30"/>
+      <x:c r="K7" s="30" t="str">
+        <x:v>Auth tests for email sign-in, Google sign-in, session/me, logout, and protected routes</x:v>
+      </x:c>
+      <x:c r="L7" s="30" t="str">
+        <x:v>wiki/product-specification/product-specification.md; wiki/api/api-specification.md</x:v>
+      </x:c>
+      <x:c r="M7" s="30" t="str">
+        <x:v>Decision: auth is required for multi-user use</x:v>
+      </x:c>
+      <x:c r="N7" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25.5" customHeight="1">
-      <x:c r="A8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Foundation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Notion Adapter</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build Notion client wrapper and adapter boundary</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-002; Notion integration access</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">All Notion calls are centralized behind service adapters with normalized errors and rate-limit awareness</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I8" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J8" s="30" t="n"/>
-      <x:c r="K8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit tests with mocked Notion client</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/tdd/tdd.md; wiki/api/api-specification.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M8" s="30" t="n"/>
-      <x:c r="N8" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A8" s="30" t="str">
+        <x:v>BE-004</x:v>
+      </x:c>
+      <x:c r="B8" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C8" s="30" t="str">
+        <x:v>Foundation</x:v>
+      </x:c>
+      <x:c r="D8" s="30" t="str">
+        <x:v>Notion Adapter</x:v>
+      </x:c>
+      <x:c r="E8" s="30" t="str">
+        <x:v>Build Notion client wrapper and adapter boundary</x:v>
+      </x:c>
+      <x:c r="F8" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G8" s="30" t="str">
+        <x:v>BE-002; Notion integration access</x:v>
+      </x:c>
+      <x:c r="H8" s="30" t="str">
+        <x:v>All Notion calls are centralized behind service adapters with normalized errors and rate-limit awareness</x:v>
+      </x:c>
+      <x:c r="I8" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J8" s="30"/>
+      <x:c r="K8" s="30" t="str">
+        <x:v>Unit tests with mocked Notion client</x:v>
+      </x:c>
+      <x:c r="L8" s="30" t="str">
+        <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md</x:v>
+      </x:c>
+      <x:c r="M8" s="30"/>
+      <x:c r="N8" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38.25" customHeight="1">
-      <x:c r="A9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-005</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Foundation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Field Mapping</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implement Notion database/property mapping contract</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Live Notion schema verification</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mappings cover app sections, Notion data sources, exact property names, live select labels, auxiliary category exclusions, and fixed workflow category rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I9" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs live Notion schema confirmation before final mapping</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Schema mapping tests and data-model update</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/database/data-model.md; wiki/tdd/tdd.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Preserve exact Notion labels in mapping; UI may use friendly display labels</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N9" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A9" s="30" t="str">
+        <x:v>BE-005</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C9" s="30" t="str">
+        <x:v>Foundation</x:v>
+      </x:c>
+      <x:c r="D9" s="30" t="str">
+        <x:v>Field Mapping</x:v>
+      </x:c>
+      <x:c r="E9" s="30" t="str">
+        <x:v>Implement Notion database/property mapping contract</x:v>
+      </x:c>
+      <x:c r="F9" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G9" s="30" t="str">
+        <x:v>Live Notion schema verification</x:v>
+      </x:c>
+      <x:c r="H9" s="30" t="str">
+        <x:v>Mappings cover app sections, Notion data sources, exact property names, live select labels, auxiliary category exclusions, and fixed workflow category rules</x:v>
+      </x:c>
+      <x:c r="I9" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J9" s="30" t="str">
+        <x:v>Needs live Notion schema confirmation before final mapping</x:v>
+      </x:c>
+      <x:c r="K9" s="30" t="str">
+        <x:v>Schema mapping tests and data-model update</x:v>
+      </x:c>
+      <x:c r="L9" s="30" t="str">
+        <x:v>wiki/database/data-model.md; wiki/tdd/tdd.md</x:v>
+      </x:c>
+      <x:c r="M9" s="30" t="str">
+        <x:v>Preserve exact Notion labels in mapping; UI may use friendly display labels</x:v>
+      </x:c>
+      <x:c r="N9" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25.5" customHeight="1">
-      <x:c r="A10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-006</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Foundation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Validation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Reject read-only, computed, hidden, and out-of-scope fields in mutations</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer, Security Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-005</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Create/update/delete payloads accept writable fields only and return VALIDATION_ERROR for forbidden fields</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I10" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J10" s="30" t="n"/>
-      <x:c r="K10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit and contract tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M10" s="30" t="n"/>
-      <x:c r="N10" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A10" s="30" t="str">
+        <x:v>BE-006</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C10" s="30" t="str">
+        <x:v>Foundation</x:v>
+      </x:c>
+      <x:c r="D10" s="30" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="E10" s="30" t="str">
+        <x:v>Reject read-only, computed, hidden, and out-of-scope fields in mutations</x:v>
+      </x:c>
+      <x:c r="F10" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer, Security Engineer</x:v>
+      </x:c>
+      <x:c r="G10" s="30" t="str">
+        <x:v>BE-005</x:v>
+      </x:c>
+      <x:c r="H10" s="30" t="str">
+        <x:v>Create/update/delete payloads accept writable fields only and return VALIDATION_ERROR for forbidden fields</x:v>
+      </x:c>
+      <x:c r="I10" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J10" s="30"/>
+      <x:c r="K10" s="30" t="str">
+        <x:v>Unit and contract tests</x:v>
+      </x:c>
+      <x:c r="L10" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
+      </x:c>
+      <x:c r="M10" s="30"/>
+      <x:c r="N10" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25.5" customHeight="1">
-      <x:c r="A11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-007</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Read</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Accounts API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build account list/detail/create/update endpoints</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-006</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Accounts support list/detail/create/update; delete marks the account inactive by setting Inactive</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I11" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J11" s="30" t="str"/>
-      <x:c r="K11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration and contract tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Decision: account records are not physically deleted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N11" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A11" s="30" t="str">
+        <x:v>BE-007</x:v>
+      </x:c>
+      <x:c r="B11" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C11" s="30" t="str">
+        <x:v>MVP Read</x:v>
+      </x:c>
+      <x:c r="D11" s="30" t="str">
+        <x:v>Accounts API</x:v>
+      </x:c>
+      <x:c r="E11" s="30" t="str">
+        <x:v>Build read-only account list/detail endpoints</x:v>
+      </x:c>
+      <x:c r="F11" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G11" s="30" t="str">
+        <x:v>BE-004; BE-006</x:v>
+      </x:c>
+      <x:c r="H11" s="30" t="str">
+        <x:v>Accounts support list/detail reads only; active-account default filtering works; current account state is returned as read-only; create/update/delete operations are absent or rejected</x:v>
+      </x:c>
+      <x:c r="I11" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J11" s="30"/>
+      <x:c r="K11" s="30" t="str">
+        <x:v>Contract tests for list/detail reads and rejected account mutations</x:v>
+      </x:c>
+      <x:c r="L11" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md; wiki/product-specification/product-specification.md</x:v>
+      </x:c>
+      <x:c r="M11" s="30" t="str">
+        <x:v>Account setup, edits, inactive marking, and deletes happen in Notion only.</x:v>
+      </x:c>
+      <x:c r="N11" s="30" t="str">
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25.5" customHeight="1">
-      <x:c r="A12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-008</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Write</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Income Categories API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build income category CRUD endpoints</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-006</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Source of Income can be created/updated; category records can be deleted according to project delete policy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I12" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J12" s="30" t="n"/>
-      <x:c r="K12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration and contract tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M12" s="30" t="n"/>
-      <x:c r="N12" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A12" s="30" t="str">
+        <x:v>BE-008</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C12" s="30" t="str">
+        <x:v>MVP Read</x:v>
+      </x:c>
+      <x:c r="D12" s="30" t="str">
+        <x:v>Income Categories API</x:v>
+      </x:c>
+      <x:c r="E12" s="30" t="str">
+        <x:v>Build read-only income category endpoints</x:v>
+      </x:c>
+      <x:c r="F12" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G12" s="30" t="str">
+        <x:v>BE-004; BE-006</x:v>
+      </x:c>
+      <x:c r="H12" s="30" t="str">
+        <x:v>Income Categories support list/detail reads for selectors, filters, category labels, and auxiliary category exclusion; create/update/delete operations are absent or rejected</x:v>
+      </x:c>
+      <x:c r="I12" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J12" s="30"/>
+      <x:c r="K12" s="30" t="str">
+        <x:v>Contract tests for list/detail reads, auxiliary category filtering support, and rejected category mutations</x:v>
+      </x:c>
+      <x:c r="L12" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md; wiki/product-specification/product-specification.md</x:v>
+      </x:c>
+      <x:c r="M12" s="30" t="str">
+        <x:v>Category maintenance stays in Notion. Normal Income choices exclude auxiliary workflow categories.</x:v>
+      </x:c>
+      <x:c r="N12" s="30" t="str">
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25.5" customHeight="1">
-      <x:c r="A13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-009</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Write</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Incomes API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build income create/read/update/soft-delete endpoints</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-006</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Income endpoints support normal income create/read/update/soft-delete and reject normal-income attempts to set transaction-only fields</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I13" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J13" s="30" t="n"/>
-      <x:c r="K13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration tests for create/edit/delete</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Transacted Account and CC Payment Covered are reserved for specialized workflows</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N13" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A13" s="30" t="str">
+        <x:v>BE-009</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>MVP Write</x:v>
+      </x:c>
+      <x:c r="D13" s="30" t="str">
+        <x:v>Incomes API</x:v>
+      </x:c>
+      <x:c r="E13" s="30" t="str">
+        <x:v>Build income create/read/update/soft-delete endpoints</x:v>
+      </x:c>
+      <x:c r="F13" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G13" s="30" t="str">
+        <x:v>BE-004; BE-006</x:v>
+      </x:c>
+      <x:c r="H13" s="30" t="str">
+        <x:v>Income endpoints support normal income create/read/update/soft-delete and reject normal-income attempts to set transaction-only fields</x:v>
+      </x:c>
+      <x:c r="I13" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J13" s="30"/>
+      <x:c r="K13" s="30" t="str">
+        <x:v>Integration tests for create/edit/delete</x:v>
+      </x:c>
+      <x:c r="L13" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
+      </x:c>
+      <x:c r="M13" s="30" t="str">
+        <x:v>Transacted Account and CC Payment Covered are reserved for specialized workflows</x:v>
+      </x:c>
+      <x:c r="N13" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25.5" customHeight="1">
-      <x:c r="A14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-010</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Write</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Transactions API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build Transfer, Credit Card Payment, Alkansya, and Receivables APIs over Incomes data source/views</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-009; view filter contract</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Workflow APIs apply fixed categories for Transfer and Credit Card Payment, include required transacted account context, and return Monthly workflow data</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I14" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J14" s="30" t="n"/>
-      <x:c r="K14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration and contract tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirm Alkansya backing view during implementation discovery</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N14" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A14" s="30" t="str">
+        <x:v>BE-010</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C14" s="30" t="str">
+        <x:v>MVP Write</x:v>
+      </x:c>
+      <x:c r="D14" s="30" t="str">
+        <x:v>Transactions API</x:v>
+      </x:c>
+      <x:c r="E14" s="30" t="str">
+        <x:v>Build Transfer, Credit Card Payment, Alkansya, and Receivables APIs over Incomes data source/views</x:v>
+      </x:c>
+      <x:c r="F14" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G14" s="30" t="str">
+        <x:v>BE-009; view filter contract</x:v>
+      </x:c>
+      <x:c r="H14" s="30" t="str">
+        <x:v>Workflow APIs apply fixed categories for Transfer and Credit Card Payment, include required transacted account context, and return Monthly workflow data</x:v>
+      </x:c>
+      <x:c r="I14" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J14" s="30"/>
+      <x:c r="K14" s="30" t="str">
+        <x:v>Integration and contract tests</x:v>
+      </x:c>
+      <x:c r="L14" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
+      </x:c>
+      <x:c r="M14" s="30" t="str">
+        <x:v>Confirm Alkansya backing view during implementation discovery</x:v>
+      </x:c>
+      <x:c r="N14" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25.5" customHeight="1">
-      <x:c r="A15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-011</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Write</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expense Categories API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build expense category CRUD endpoints</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-006</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Categories, Monthly Budget, Upcoming Budget, and Auxiliary are writable; category delete follows project policy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I15" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J15" s="30" t="n"/>
-      <x:c r="K15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration and contract tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M15" s="30" t="n"/>
-      <x:c r="N15" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A15" s="30" t="str">
+        <x:v>BE-011</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C15" s="30" t="str">
+        <x:v>MVP Read</x:v>
+      </x:c>
+      <x:c r="D15" s="30" t="str">
+        <x:v>Expense Categories API</x:v>
+      </x:c>
+      <x:c r="E15" s="30" t="str">
+        <x:v>Build read-only expense category endpoints</x:v>
+      </x:c>
+      <x:c r="F15" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G15" s="30" t="str">
+        <x:v>BE-004; BE-006</x:v>
+      </x:c>
+      <x:c r="H15" s="30" t="str">
+        <x:v>Expense Categories support list/detail reads for selectors, filters, auxiliary flags, monthly budget, upcoming budget, and category reporting config; create/update/delete operations are absent or rejected</x:v>
+      </x:c>
+      <x:c r="I15" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J15" s="30"/>
+      <x:c r="K15" s="30" t="str">
+        <x:v>Contract tests for list/detail reads, budget/config fields, and rejected category mutations</x:v>
+      </x:c>
+      <x:c r="L15" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md; wiki/product-specification/product-specification.md</x:v>
+      </x:c>
+      <x:c r="M15" s="30" t="str">
+        <x:v>Category maintenance stays in Notion. App-calculated category reporting uses scoped Expense records plus budget config.</x:v>
+      </x:c>
+      <x:c r="N15" s="30" t="str">
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38.25" customHeight="1">
-      <x:c r="A16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-012</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Write</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expenses API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build expense create/read/update/soft-delete endpoints</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-006</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expense endpoints support required view modes and validate conditional field groups for credit-card and Pasabuy flows</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I16" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J16" s="30" t="n"/>
-      <x:c r="K16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration tests for create/edit/delete</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Credit-card fields require Credit Account or BYPL account context; Pasabuy fields require Pasabuy flow/category</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N16" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A16" s="30" t="str">
+        <x:v>BE-012</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C16" s="30" t="str">
+        <x:v>MVP Write</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="str">
+        <x:v>Expenses API</x:v>
+      </x:c>
+      <x:c r="E16" s="30" t="str">
+        <x:v>Build expense create/read/update/soft-delete endpoints</x:v>
+      </x:c>
+      <x:c r="F16" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G16" s="30" t="str">
+        <x:v>BE-004; BE-006</x:v>
+      </x:c>
+      <x:c r="H16" s="30" t="str">
+        <x:v>Expense endpoints support required view modes and validate conditional field groups for credit-card and Pasabuy flows</x:v>
+      </x:c>
+      <x:c r="I16" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J16" s="30"/>
+      <x:c r="K16" s="30" t="str">
+        <x:v>Integration tests for create/edit/delete</x:v>
+      </x:c>
+      <x:c r="L16" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
+      </x:c>
+      <x:c r="M16" s="30" t="str">
+        <x:v>Credit-card fields require Credit Account or BYPL account context; Pasabuy fields require Pasabuy flow/category</x:v>
+      </x:c>
+      <x:c r="N16" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25.5" customHeight="1">
-      <x:c r="A17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-013</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Write</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expense Scheduler API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build scheduler workflows over Expenses data source/views</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-012; view filter contract</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Scheduler endpoints reuse expense mapping and delete behavior while exposing to-buy, to-pay, installment, and scheduled workflows</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I17" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J17" s="30" t="n"/>
-      <x:c r="K17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration and contract tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No separate canonical scheduler database</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N17" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A17" s="30" t="str">
+        <x:v>BE-013</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C17" s="30" t="str">
+        <x:v>MVP Write</x:v>
+      </x:c>
+      <x:c r="D17" s="30" t="str">
+        <x:v>Expense Scheduler API</x:v>
+      </x:c>
+      <x:c r="E17" s="30" t="str">
+        <x:v>Build scheduler workflows over Expenses data source/views</x:v>
+      </x:c>
+      <x:c r="F17" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G17" s="30" t="str">
+        <x:v>BE-012; view filter contract</x:v>
+      </x:c>
+      <x:c r="H17" s="30" t="str">
+        <x:v>Scheduler endpoints reuse expense mapping and delete behavior while exposing to-buy, to-pay, installment, and scheduled workflows</x:v>
+      </x:c>
+      <x:c r="I17" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J17" s="30"/>
+      <x:c r="K17" s="30" t="str">
+        <x:v>Integration and contract tests</x:v>
+      </x:c>
+      <x:c r="L17" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
+      </x:c>
+      <x:c r="M17" s="30" t="str">
+        <x:v>No separate canonical scheduler database</x:v>
+      </x:c>
+      <x:c r="N17" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25.5" customHeight="1">
-      <x:c r="A18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-014</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Read</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sync Pull</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build pull-latest data normalization</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-005</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend pulls latest app-scoped Notion data, normalizes it into app DTOs, and includes computed/read-only values in responses</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I18" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J18" s="30" t="n"/>
-      <x:c r="K18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration tests with mocked Notion pages</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/tdd/tdd.md; wiki/api/api-specification.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M18" s="30" t="n"/>
-      <x:c r="N18" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A18" s="30" t="str">
+        <x:v>BE-014</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C18" s="30" t="str">
+        <x:v>MVP Read</x:v>
+      </x:c>
+      <x:c r="D18" s="30" t="str">
+        <x:v>Sync Pull</x:v>
+      </x:c>
+      <x:c r="E18" s="30" t="str">
+        <x:v>Build pull-latest data normalization</x:v>
+      </x:c>
+      <x:c r="F18" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G18" s="30" t="str">
+        <x:v>BE-004; BE-005</x:v>
+      </x:c>
+      <x:c r="H18" s="30" t="str">
+        <x:v>Backend pulls latest app-scoped Notion data, normalizes it into app DTOs, and includes computed/read-only values in responses</x:v>
+      </x:c>
+      <x:c r="I18" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J18" s="30"/>
+      <x:c r="K18" s="30" t="str">
+        <x:v>Integration tests with mocked Notion pages</x:v>
+      </x:c>
+      <x:c r="L18" s="30" t="str">
+        <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md</x:v>
+      </x:c>
+      <x:c r="M18" s="30"/>
+      <x:c r="N18" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25.5" customHeight="1">
-      <x:c r="A19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-015</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Write</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sync Commit</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build queued sync commit orchestration</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-014; metadata store contract</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sync commit validates operations, writes to Notion, handles partial failure, pulls fresh snapshot, and returns applied/failed results</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I19" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J19" s="30" t="n"/>
-      <x:c r="K19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration and contract tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/tdd/tdd.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M19" s="30" t="n"/>
-      <x:c r="N19" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A19" s="30" t="str">
+        <x:v>BE-015</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C19" s="30" t="str">
+        <x:v>MVP Write</x:v>
+      </x:c>
+      <x:c r="D19" s="30" t="str">
+        <x:v>Sync Commit</x:v>
+      </x:c>
+      <x:c r="E19" s="30" t="str">
+        <x:v>Build queued sync commit orchestration</x:v>
+      </x:c>
+      <x:c r="F19" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G19" s="30" t="str">
+        <x:v>BE-014; metadata store contract</x:v>
+      </x:c>
+      <x:c r="H19" s="30" t="str">
+        <x:v>Sync commit validates operations, writes to Notion, handles partial failure, pulls fresh snapshot, and returns applied/failed results</x:v>
+      </x:c>
+      <x:c r="I19" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J19" s="30"/>
+      <x:c r="K19" s="30" t="str">
+        <x:v>Integration and contract tests</x:v>
+      </x:c>
+      <x:c r="L19" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/tdd/tdd.md</x:v>
+      </x:c>
+      <x:c r="M19" s="30"/>
+      <x:c r="N19" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="38.25" customHeight="1">
-      <x:c r="A20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-016</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Foundation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Metadata Store</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Design and implement supporting metadata store</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Storage decision</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PostgreSQL supports sync logs, pending mutations, conflicts, audit events, sessions if needed, and cached snapshots without becoming finance source of truth</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I20" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J20" s="30" t="str"/>
-      <x:c r="K20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Data model docs and PostgreSQL persistence tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/database/data-model.md; wiki/tdd/tdd.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Decision: PostgreSQL is primary durable metadata storage; Redis is optional for cache, rate limits, sessions, or queue coordination</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N20" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A20" s="30" t="str">
+        <x:v>BE-016</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C20" s="30" t="str">
+        <x:v>Foundation</x:v>
+      </x:c>
+      <x:c r="D20" s="30" t="str">
+        <x:v>Metadata Store</x:v>
+      </x:c>
+      <x:c r="E20" s="30" t="str">
+        <x:v>Design and implement supporting metadata store</x:v>
+      </x:c>
+      <x:c r="F20" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G20" s="30" t="str">
+        <x:v>Storage decision</x:v>
+      </x:c>
+      <x:c r="H20" s="30" t="str">
+        <x:v>PostgreSQL supports sync logs, pending mutations, conflicts, audit events, sessions if needed, and cached snapshots without becoming finance source of truth</x:v>
+      </x:c>
+      <x:c r="I20" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J20" s="30"/>
+      <x:c r="K20" s="30" t="str">
+        <x:v>Data model docs and PostgreSQL persistence tests</x:v>
+      </x:c>
+      <x:c r="L20" s="30" t="str">
+        <x:v>wiki/database/data-model.md; wiki/tdd/tdd.md</x:v>
+      </x:c>
+      <x:c r="M20" s="30" t="str">
+        <x:v>Decision: PostgreSQL is primary durable metadata storage; Redis is optional for cache, rate limits, sessions, or queue coordination</x:v>
+      </x:c>
+      <x:c r="N20" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25.5" customHeight="1">
-      <x:c r="A21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-017</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hardening</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Conflict Detection</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detect stale edits and conflicts</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-014; metadata snapshots</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend detects records changed in Notion after app load and returns CONFLICT_ERROR with user-safe details</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I21" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J21" s="30" t="n"/>
-      <x:c r="K21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Integration tests with stale last-edited metadata</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/tdd/tdd.md; wiki/api/api-specification.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M21" s="30" t="n"/>
-      <x:c r="N21" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A21" s="30" t="str">
+        <x:v>BE-017</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>Hardening</x:v>
+      </x:c>
+      <x:c r="D21" s="30" t="str">
+        <x:v>Conflict Detection</x:v>
+      </x:c>
+      <x:c r="E21" s="30" t="str">
+        <x:v>Detect stale edits and conflicts</x:v>
+      </x:c>
+      <x:c r="F21" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G21" s="30" t="str">
+        <x:v>BE-014; metadata snapshots</x:v>
+      </x:c>
+      <x:c r="H21" s="30" t="str">
+        <x:v>Backend detects records changed in Notion after app load and returns CONFLICT_ERROR with user-safe details</x:v>
+      </x:c>
+      <x:c r="I21" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J21" s="30"/>
+      <x:c r="K21" s="30" t="str">
+        <x:v>Integration tests with stale last-edited metadata</x:v>
+      </x:c>
+      <x:c r="L21" s="30" t="str">
+        <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md</x:v>
+      </x:c>
+      <x:c r="M21" s="30"/>
+      <x:c r="N21" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="38.25" customHeight="1">
-      <x:c r="A22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-018</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hardening</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Schema Drift</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implement schema health and drift checks</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-005; BE-004</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">System verifies data sources, properties, property types, relation targets, and select/status options; schema drift returns SCHEMA_DRIFT_DETECTED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I22" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J22" s="30" t="n"/>
-      <x:c r="K22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Schema status integration tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/tdd/tdd.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M22" s="30" t="n"/>
-      <x:c r="N22" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A22" s="30" t="str">
+        <x:v>BE-018</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C22" s="30" t="str">
+        <x:v>Hardening</x:v>
+      </x:c>
+      <x:c r="D22" s="30" t="str">
+        <x:v>Schema Drift</x:v>
+      </x:c>
+      <x:c r="E22" s="30" t="str">
+        <x:v>Implement schema health and drift checks</x:v>
+      </x:c>
+      <x:c r="F22" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G22" s="30" t="str">
+        <x:v>BE-005; BE-004</x:v>
+      </x:c>
+      <x:c r="H22" s="30" t="str">
+        <x:v>System verifies data sources, properties, property types, relation targets, and select/status options; schema drift returns SCHEMA_DRIFT_DETECTED</x:v>
+      </x:c>
+      <x:c r="I22" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J22" s="30"/>
+      <x:c r="K22" s="30" t="str">
+        <x:v>Schema status integration tests</x:v>
+      </x:c>
+      <x:c r="L22" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/tdd/tdd.md</x:v>
+      </x:c>
+      <x:c r="M22" s="30"/>
+      <x:c r="N22" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25.5" customHeight="1">
-      <x:c r="A23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-019</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hardening</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Error Normalization</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Normalize validation, Notion, access, rate-limit, conflict, and schema errors</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer, Security Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-006; BE-017; BE-018</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">API returns stable error codes and user-safe messages without raw stack traces, tokens, or sensitive finance payloads</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I23" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J23" s="30" t="n"/>
-      <x:c r="K23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Contract and security tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/tdd/tdd.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M23" s="30" t="n"/>
-      <x:c r="N23" s="30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A23" s="30" t="str">
+        <x:v>BE-019</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>Hardening</x:v>
+      </x:c>
+      <x:c r="D23" s="30" t="str">
+        <x:v>Error Normalization</x:v>
+      </x:c>
+      <x:c r="E23" s="30" t="str">
+        <x:v>Normalize validation, Notion, access, rate-limit, conflict, and schema errors</x:v>
+      </x:c>
+      <x:c r="F23" s="30" t="str">
+        <x:v>Backend &amp; Database Engineer, Security Engineer</x:v>
+      </x:c>
+      <x:c r="G23" s="30" t="str">
+        <x:v>BE-004; BE-006; BE-017; BE-018</x:v>
+      </x:c>
+      <x:c r="H23" s="30" t="str">
+        <x:v>API returns stable error codes and user-safe messages without raw stack traces, tokens, or sensitive finance payloads</x:v>
+      </x:c>
+      <x:c r="I23" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J23" s="30"/>
+      <x:c r="K23" s="30" t="str">
+        <x:v>Contract and security tests</x:v>
+      </x:c>
+      <x:c r="L23" s="30" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/tdd/tdd.md</x:v>
+      </x:c>
+      <x:c r="M23" s="30"/>
+      <x:c r="N23" s="30" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="25.5" customHeight="1">
-      <x:c r="A24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-020</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hardening</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Logging and Audit</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implement redacted operational logging and audit events</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer, Security Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-016; BE-019</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Production logs redact sensitive finance payloads and credentials while preserving useful sync/error/audit metadata</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I24" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J24" s="6" t="n"/>
-      <x:c r="K24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Security review and log redaction tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/database/data-model.md; wiki/tdd/tdd.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M24" s="6" t="n"/>
-      <x:c r="N24" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A24" s="6" t="str">
+        <x:v>BE-020</x:v>
+      </x:c>
+      <x:c r="B24" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C24" s="6" t="str">
+        <x:v>Hardening</x:v>
+      </x:c>
+      <x:c r="D24" s="6" t="str">
+        <x:v>Logging and Audit</x:v>
+      </x:c>
+      <x:c r="E24" s="6" t="str">
+        <x:v>Implement redacted operational logging and audit events</x:v>
+      </x:c>
+      <x:c r="F24" s="6" t="str">
+        <x:v>Backend &amp; Database Engineer, Security Engineer</x:v>
+      </x:c>
+      <x:c r="G24" s="6" t="str">
+        <x:v>BE-016; BE-019</x:v>
+      </x:c>
+      <x:c r="H24" s="6" t="str">
+        <x:v>Production logs redact sensitive finance payloads and credentials while preserving useful sync/error/audit metadata</x:v>
+      </x:c>
+      <x:c r="I24" s="13" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J24" s="6"/>
+      <x:c r="K24" s="6" t="str">
+        <x:v>Security review and log redaction tests</x:v>
+      </x:c>
+      <x:c r="L24" s="6" t="str">
+        <x:v>wiki/database/data-model.md; wiki/tdd/tdd.md</x:v>
+      </x:c>
+      <x:c r="M24" s="6"/>
+      <x:c r="N24" s="6" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-021</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MVP Read</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Monthly Monitoring API</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build read-only Monthly Monitoring endpoints</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Backend &amp; Database Engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE-004; BE-005</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GET monthly monitoring endpoints return read-only month-level monitoring data with related income and expense category context; mutation endpoints are absent or forbidden</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I25" s="25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J25" s="6" t="n"/>
-      <x:c r="K25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">API integration and contract test results</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wiki/api/api-specification.md; wiki/database/data-model.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Do not expose edit paths for Monthly Monitoring normal app flows</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N25" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-03</x:t>
-        </x:is>
+      <x:c r="A25" s="6" t="str">
+        <x:v>BE-021</x:v>
+      </x:c>
+      <x:c r="B25" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="str">
+        <x:v>MVP Read</x:v>
+      </x:c>
+      <x:c r="D25" s="6" t="str">
+        <x:v>Monthly Monitoring API</x:v>
+      </x:c>
+      <x:c r="E25" s="6" t="str">
+        <x:v>Build read-only Monthly Monitoring endpoints</x:v>
+      </x:c>
+      <x:c r="F25" s="6" t="str">
+        <x:v>Backend &amp; Database Engineer</x:v>
+      </x:c>
+      <x:c r="G25" s="6" t="str">
+        <x:v>BE-004; BE-005</x:v>
+      </x:c>
+      <x:c r="H25" s="6" t="str">
+        <x:v>GET monthly monitoring endpoints return read-only month-level monitoring data with related income and expense category context; mutation endpoints are absent or forbidden</x:v>
+      </x:c>
+      <x:c r="I25" s="25" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="J25" s="6"/>
+      <x:c r="K25" s="6" t="str">
+        <x:v>API integration and contract test results</x:v>
+      </x:c>
+      <x:c r="L25" s="6" t="str">
+        <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
+      </x:c>
+      <x:c r="M25" s="6" t="str">
+        <x:v>Do not expose edit paths for Monthly Monitoring normal app flows</x:v>
+      </x:c>
+      <x:c r="N25" s="6" t="str">
+        <x:v>2026-07-03</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
1st backend impl push
</commit_message>
<xml_diff>
--- a/wiki/development-plan/notion-finance-development-plan.xlsx
+++ b/wiki/development-plan/notion-finance-development-plan.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf46e0e4d0d894d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frontend-dev-plan" sheetId="2" r:id="R285227dcec9a444b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backend-dev-plan" sheetId="3" r:id="Rf1327151e5244157"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="integration-dev-plan" sheetId="4" r:id="R10b6a63a6bef4834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="testing-dev-plan" sheetId="5" r:id="Re060937ae05c4d3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd2dce6ff46084b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frontend-dev-plan" sheetId="2" r:id="R9c4b330be33148f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backend-dev-plan" sheetId="3" r:id="R560789388da241a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="integration-dev-plan" sheetId="4" r:id="Rc21013fc8c9a4285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="testing-dev-plan" sheetId="5" r:id="R577f25f1759f4b63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -706,7 +706,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="17" t="str">
-        <x:v>Updated 2026-07-04. Backend plan is aligned to the current read-only Accounts, Income Categories, and Expense Categories design while frontend implementation remains in progress and Notion remains the source of truth.</x:v>
+        <x:v>Updated 2026-07-04. Backend foundation now includes NestJS route modules, configuration, mapping, validation, sync, schema status, dashboard/monthly monitoring responses, and backend tests over a development Notion-shaped repository. Live Notion writes, live schema checks, PostgreSQL persistence, and production auth remain pending.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -796,16 +796,16 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="C6" s="8" t="n">
-        <x:v>21</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E6" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F6" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G6" s="8" t="n">
         <x:v>0</x:v>
@@ -1001,7 +1001,7 @@
         </x:is>
       </x:c>
       <x:c r="E16" s="30" t="str">
-        <x:v>Document duplicated Notion access details, confirm compact/detail fields, and confirm live relation/category mappings during backend implementation discovery.</x:v>
+        <x:v>Replace the development repository with the live Notion adapter, confirm live schema/property mappings, then add PostgreSQL persistence for sync/audit/conflict metadata.</x:v>
       </x:c>
       <x:c r="F16" s="30" t="n"/>
       <x:c r="G16" s="30" t="n"/>
@@ -2538,19 +2538,17 @@
         <x:v>NestJS service exists under service/ with health endpoint, scripts, lint/typecheck/test placeholders, and environment loading baseline</x:v>
       </x:c>
       <x:c r="I5" s="13" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="J5" s="4" t="str">
-        <x:v>Pending explicit backend implementation request</x:v>
-      </x:c>
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="J5" s="4"/>
       <x:c r="K5" s="4" t="str">
-        <x:v>Build/lint/typecheck commands pass once tooling exists</x:v>
+        <x:v>Backend verification passed on 2026-07-04: npm --prefix service run typecheck; npm --prefix service run test; npm --prefix service run build. NestJS service scaffold, health endpoint, package scripts, config baseline, and README exist under service/.</x:v>
       </x:c>
       <x:c r="L5" s="4" t="str">
         <x:v>wiki/project-structure/project-structure.md; wiki/tdd/tdd.md</x:v>
       </x:c>
       <x:c r="M5" s="4" t="str">
-        <x:v>Do this only after backend implementation approval.</x:v>
+        <x:v>Foundation implemented with a development Notion-shaped repository; live integration remains separate work.</x:v>
       </x:c>
       <x:c r="N5" s="4" t="str">
         <x:v>2026-07-04</x:v>
@@ -2582,20 +2580,20 @@
         <x:v>Notion token, database IDs, metadata store settings, and environment-specific options are read server-side only and validated on startup</x:v>
       </x:c>
       <x:c r="I6" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J6" s="30"/>
       <x:c r="K6" s="30" t="str">
-        <x:v>Unit tests and secret scan</x:v>
+        <x:v>Server-side config module and service/.env.example are in place; startup validation and production secret hardening remain.</x:v>
       </x:c>
       <x:c r="L6" s="30" t="str">
         <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
       </x:c>
       <x:c r="M6" s="30" t="str">
-        <x:v>Do not expose token or server-only env values to application/</x:v>
+        <x:v>Notion secrets stay server-side; no frontend token exposure.</x:v>
       </x:c>
       <x:c r="N6" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25.5" customHeight="1">
@@ -2624,20 +2622,20 @@
         <x:v>Email sign-in and Google sign-in are implemented; write endpoints and sync commit are protected</x:v>
       </x:c>
       <x:c r="I7" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J7" s="30"/>
       <x:c r="K7" s="30" t="str">
-        <x:v>Auth tests for email sign-in, Google sign-in, session/me, logout, and protected routes</x:v>
+        <x:v>Development auth shell endpoints exist for login, Google placeholder, me, and logout.</x:v>
       </x:c>
       <x:c r="L7" s="30" t="str">
         <x:v>wiki/product-specification/product-specification.md; wiki/api/api-specification.md</x:v>
       </x:c>
       <x:c r="M7" s="30" t="str">
-        <x:v>Decision: auth is required for multi-user use</x:v>
+        <x:v>Production email/Google auth and route protection are not complete.</x:v>
       </x:c>
       <x:c r="N7" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25.5" customHeight="1">
@@ -2666,18 +2664,20 @@
         <x:v>All Notion calls are centralized behind service adapters with normalized errors and rate-limit awareness</x:v>
       </x:c>
       <x:c r="I8" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J8" s="30"/>
       <x:c r="K8" s="30" t="str">
-        <x:v>Unit tests with mocked Notion client</x:v>
+        <x:v>NotionService now centralizes the adapter boundary with normalized development data operations.</x:v>
       </x:c>
       <x:c r="L8" s="30" t="str">
         <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md</x:v>
       </x:c>
-      <x:c r="M8" s="30"/>
+      <x:c r="M8" s="30" t="str">
+        <x:v>Live Notion client calls, retry/rate-limit behavior, and provider error mapping remain.</x:v>
+      </x:c>
       <x:c r="N8" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38.25" customHeight="1">
@@ -2706,22 +2706,22 @@
         <x:v>Mappings cover app sections, Notion data sources, exact property names, live select labels, auxiliary category exclusions, and fixed workflow category rules</x:v>
       </x:c>
       <x:c r="I9" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J9" s="30" t="str">
-        <x:v>Needs live Notion schema confirmation before final mapping</x:v>
+        <x:v>Needs live Notion schema confirmation before final mapping.</x:v>
       </x:c>
       <x:c r="K9" s="30" t="str">
-        <x:v>Schema mapping tests and data-model update</x:v>
+        <x:v>MappingService defines app resource mappings and fixed workflow category rules against the documented design.</x:v>
       </x:c>
       <x:c r="L9" s="30" t="str">
         <x:v>wiki/database/data-model.md; wiki/tdd/tdd.md</x:v>
       </x:c>
       <x:c r="M9" s="30" t="str">
-        <x:v>Preserve exact Notion labels in mapping; UI may use friendly display labels</x:v>
+        <x:v>Exact live property IDs/types/options still need verification against the duplicated Notion workspace.</x:v>
       </x:c>
       <x:c r="N9" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25.5" customHeight="1">
@@ -2750,18 +2750,20 @@
         <x:v>Create/update/delete payloads accept writable fields only and return VALIDATION_ERROR for forbidden fields</x:v>
       </x:c>
       <x:c r="I10" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="J10" s="30"/>
       <x:c r="K10" s="30" t="str">
-        <x:v>Unit and contract tests</x:v>
+        <x:v>Backend verification passed on 2026-07-04: npm --prefix service run typecheck; npm --prefix service run test; npm --prefix service run build. Validation tests cover read-only/computed/out-of-scope field rejection and workflow category overrides.</x:v>
       </x:c>
       <x:c r="L10" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
       </x:c>
-      <x:c r="M10" s="30"/>
+      <x:c r="M10" s="30" t="str">
+        <x:v>Validation runs before development repository mutations and sync commit operations.</x:v>
+      </x:c>
       <x:c r="N10" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25.5" customHeight="1">
@@ -2790,17 +2792,17 @@
         <x:v>Accounts support list/detail reads only; active-account default filtering works; current account state is returned as read-only; create/update/delete operations are absent or rejected</x:v>
       </x:c>
       <x:c r="I11" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="J11" s="30"/>
       <x:c r="K11" s="30" t="str">
-        <x:v>Contract tests for list/detail reads and rejected account mutations</x:v>
+        <x:v>Backend verification passed on 2026-07-04: npm --prefix service run typecheck; npm --prefix service run test; npm --prefix service run build. Accounts list/detail reads and default active-account filtering are implemented; sync rejects account mutations.</x:v>
       </x:c>
       <x:c r="L11" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md; wiki/product-specification/product-specification.md</x:v>
       </x:c>
       <x:c r="M11" s="30" t="str">
-        <x:v>Account setup, edits, inactive marking, and deletes happen in Notion only.</x:v>
+        <x:v>Account setup and edits remain Notion-only.</x:v>
       </x:c>
       <x:c r="N11" s="30" t="str">
         <x:v>2026-07-04</x:v>
@@ -2832,17 +2834,17 @@
         <x:v>Income Categories support list/detail reads for selectors, filters, category labels, and auxiliary category exclusion; create/update/delete operations are absent or rejected</x:v>
       </x:c>
       <x:c r="I12" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="J12" s="30"/>
       <x:c r="K12" s="30" t="str">
-        <x:v>Contract tests for list/detail reads, auxiliary category filtering support, and rejected category mutations</x:v>
+        <x:v>Backend verification passed on 2026-07-04: npm --prefix service run typecheck; npm --prefix service run test; npm --prefix service run build. Income category list/detail reads and auxiliary-category exclusion support are implemented; sync rejects category mutations.</x:v>
       </x:c>
       <x:c r="L12" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md; wiki/product-specification/product-specification.md</x:v>
       </x:c>
       <x:c r="M12" s="30" t="str">
-        <x:v>Category maintenance stays in Notion. Normal Income choices exclude auxiliary workflow categories.</x:v>
+        <x:v>Income category maintenance remains Notion-only.</x:v>
       </x:c>
       <x:c r="N12" s="30" t="str">
         <x:v>2026-07-04</x:v>
@@ -2874,20 +2876,20 @@
         <x:v>Income endpoints support normal income create/read/update/soft-delete and reject normal-income attempts to set transaction-only fields</x:v>
       </x:c>
       <x:c r="I13" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J13" s="30"/>
       <x:c r="K13" s="30" t="str">
-        <x:v>Integration tests for create/edit/delete</x:v>
+        <x:v>Income CRUD and soft-delete endpoint surface exists over the development repository.</x:v>
       </x:c>
       <x:c r="L13" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
       </x:c>
       <x:c r="M13" s="30" t="str">
-        <x:v>Transacted Account and CC Payment Covered are reserved for specialized workflows</x:v>
+        <x:v>Live Notion create/update/soft-delete writes remain.</x:v>
       </x:c>
       <x:c r="N13" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25.5" customHeight="1">
@@ -2916,20 +2918,20 @@
         <x:v>Workflow APIs apply fixed categories for Transfer and Credit Card Payment, include required transacted account context, and return Monthly workflow data</x:v>
       </x:c>
       <x:c r="I14" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J14" s="30"/>
       <x:c r="K14" s="30" t="str">
-        <x:v>Integration and contract tests</x:v>
+        <x:v>Transactions, Transfer, Credit Card Payment, Alkansya, and Receivables controllers exist with fixed category validation.</x:v>
       </x:c>
       <x:c r="L14" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
       </x:c>
       <x:c r="M14" s="30" t="str">
-        <x:v>Confirm Alkansya backing view during implementation discovery</x:v>
+        <x:v>Live view filters, Notion-backed workflow mapping, and Alkansya backing confirmation remain.</x:v>
       </x:c>
       <x:c r="N14" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25.5" customHeight="1">
@@ -2958,17 +2960,17 @@
         <x:v>Expense Categories support list/detail reads for selectors, filters, auxiliary flags, monthly budget, upcoming budget, and category reporting config; create/update/delete operations are absent or rejected</x:v>
       </x:c>
       <x:c r="I15" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="J15" s="30"/>
       <x:c r="K15" s="30" t="str">
-        <x:v>Contract tests for list/detail reads, budget/config fields, and rejected category mutations</x:v>
+        <x:v>Backend verification passed on 2026-07-04: npm --prefix service run typecheck; npm --prefix service run test; npm --prefix service run build. Expense category list/detail reads expose budget/config fields; sync rejects category mutations.</x:v>
       </x:c>
       <x:c r="L15" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md; wiki/product-specification/product-specification.md</x:v>
       </x:c>
       <x:c r="M15" s="30" t="str">
-        <x:v>Category maintenance stays in Notion. App-calculated category reporting uses scoped Expense records plus budget config.</x:v>
+        <x:v>Expense category maintenance remains Notion-only.</x:v>
       </x:c>
       <x:c r="N15" s="30" t="str">
         <x:v>2026-07-04</x:v>
@@ -3000,20 +3002,20 @@
         <x:v>Expense endpoints support required view modes and validate conditional field groups for credit-card and Pasabuy flows</x:v>
       </x:c>
       <x:c r="I16" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30" t="str">
-        <x:v>Integration tests for create/edit/delete</x:v>
+        <x:v>Expense CRUD and soft-delete endpoint surface exists over the development repository.</x:v>
       </x:c>
       <x:c r="L16" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
       </x:c>
       <x:c r="M16" s="30" t="str">
-        <x:v>Credit-card fields require Credit Account or BYPL account context; Pasabuy fields require Pasabuy flow/category</x:v>
+        <x:v>Live Notion writes plus stronger conditional relation validation remain.</x:v>
       </x:c>
       <x:c r="N16" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25.5" customHeight="1">
@@ -3042,20 +3044,20 @@
         <x:v>Scheduler endpoints reuse expense mapping and delete behavior while exposing to-buy, to-pay, installment, and scheduled workflows</x:v>
       </x:c>
       <x:c r="I17" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J17" s="30"/>
       <x:c r="K17" s="30" t="str">
-        <x:v>Integration and contract tests</x:v>
+        <x:v>Expense Scheduler controller/module exists over the development repository.</x:v>
       </x:c>
       <x:c r="L17" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
       </x:c>
       <x:c r="M17" s="30" t="str">
-        <x:v>No separate canonical scheduler database</x:v>
+        <x:v>Live scheduler view filters and Notion-backed workflow behavior remain.</x:v>
       </x:c>
       <x:c r="N17" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25.5" customHeight="1">
@@ -3084,18 +3086,20 @@
         <x:v>Backend pulls latest app-scoped Notion data, normalizes it into app DTOs, and includes computed/read-only values in responses</x:v>
       </x:c>
       <x:c r="I18" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J18" s="30"/>
       <x:c r="K18" s="30" t="str">
-        <x:v>Integration tests with mocked Notion pages</x:v>
+        <x:v>Sync pull returns scoped snapshots from the development repository.</x:v>
       </x:c>
       <x:c r="L18" s="30" t="str">
         <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md</x:v>
       </x:c>
-      <x:c r="M18" s="30"/>
+      <x:c r="M18" s="30" t="str">
+        <x:v>Live Notion pull normalization and pagination remain.</x:v>
+      </x:c>
       <x:c r="N18" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25.5" customHeight="1">
@@ -3124,18 +3128,20 @@
         <x:v>Sync commit validates operations, writes to Notion, handles partial failure, pulls fresh snapshot, and returns applied/failed results</x:v>
       </x:c>
       <x:c r="I19" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J19" s="30"/>
       <x:c r="K19" s="30" t="str">
-        <x:v>Integration and contract tests</x:v>
+        <x:v>Sync commit validates operations, returns applied/failed results, and can return fresh development snapshots.</x:v>
       </x:c>
       <x:c r="L19" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/tdd/tdd.md</x:v>
       </x:c>
-      <x:c r="M19" s="30"/>
+      <x:c r="M19" s="30" t="str">
+        <x:v>Live Notion write orchestration, retry behavior, and post-write pull from Notion remain.</x:v>
+      </x:c>
       <x:c r="N19" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="38.25" customHeight="1">
@@ -3164,20 +3170,20 @@
         <x:v>PostgreSQL supports sync logs, pending mutations, conflicts, audit events, sessions if needed, and cached snapshots without becoming finance source of truth</x:v>
       </x:c>
       <x:c r="I20" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J20" s="30"/>
       <x:c r="K20" s="30" t="str">
-        <x:v>Data model docs and PostgreSQL persistence tests</x:v>
+        <x:v>In-memory metadata and audit baseline services exist.</x:v>
       </x:c>
       <x:c r="L20" s="30" t="str">
         <x:v>wiki/database/data-model.md; wiki/tdd/tdd.md</x:v>
       </x:c>
       <x:c r="M20" s="30" t="str">
-        <x:v>Decision: PostgreSQL is primary durable metadata storage; Redis is optional for cache, rate limits, sessions, or queue coordination</x:v>
+        <x:v>PostgreSQL schema, migrations, repository layer, and durable persistence remain.</x:v>
       </x:c>
       <x:c r="N20" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25.5" customHeight="1">
@@ -3206,18 +3212,20 @@
         <x:v>Backend detects records changed in Notion after app load and returns CONFLICT_ERROR with user-safe details</x:v>
       </x:c>
       <x:c r="I21" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J21" s="30"/>
       <x:c r="K21" s="30" t="str">
-        <x:v>Integration tests with stale last-edited metadata</x:v>
+        <x:v>Conflict service baseline exists.</x:v>
       </x:c>
       <x:c r="L21" s="30" t="str">
         <x:v>wiki/tdd/tdd.md; wiki/api/api-specification.md</x:v>
       </x:c>
-      <x:c r="M21" s="30"/>
+      <x:c r="M21" s="30" t="str">
+        <x:v>Conflict checks still need Notion last-edited metadata, cached snapshots, and endpoint integration.</x:v>
+      </x:c>
       <x:c r="N21" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="38.25" customHeight="1">
@@ -3246,18 +3254,22 @@
         <x:v>System verifies data sources, properties, property types, relation targets, and select/status options; schema drift returns SCHEMA_DRIFT_DETECTED</x:v>
       </x:c>
       <x:c r="I22" s="13" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="J22" s="30"/>
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J22" s="30" t="str">
+        <x:v>Blocked on Notion credentials and duplicated workspace schema access.</x:v>
+      </x:c>
       <x:c r="K22" s="30" t="str">
-        <x:v>Schema status integration tests</x:v>
+        <x:v>Schema-status endpoint reports configuration/mapping status and identifies when live Notion validation is unavailable.</x:v>
       </x:c>
       <x:c r="L22" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/tdd/tdd.md</x:v>
       </x:c>
-      <x:c r="M22" s="30"/>
+      <x:c r="M22" s="30" t="str">
+        <x:v>Live schema checks for data sources, property types, relation targets, and select options remain.</x:v>
+      </x:c>
       <x:c r="N22" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25.5" customHeight="1">
@@ -3286,18 +3298,20 @@
         <x:v>API returns stable error codes and user-safe messages without raw stack traces, tokens, or sensitive finance payloads</x:v>
       </x:c>
       <x:c r="I23" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J23" s="30"/>
       <x:c r="K23" s="30" t="str">
-        <x:v>Contract and security tests</x:v>
+        <x:v>Global exception filter normalizes HTTP errors and hides raw non-HTTP exception details.</x:v>
       </x:c>
       <x:c r="L23" s="30" t="str">
         <x:v>wiki/api/api-specification.md; wiki/tdd/tdd.md</x:v>
       </x:c>
-      <x:c r="M23" s="30"/>
+      <x:c r="M23" s="30" t="str">
+        <x:v>Notion, rate-limit, access, conflict, and schema-error normalization remain.</x:v>
+      </x:c>
       <x:c r="N23" s="30" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="25.5" customHeight="1">
@@ -3326,18 +3340,20 @@
         <x:v>Production logs redact sensitive finance payloads and credentials while preserving useful sync/error/audit metadata</x:v>
       </x:c>
       <x:c r="I24" s="13" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J24" s="6"/>
       <x:c r="K24" s="6" t="str">
-        <x:v>Security review and log redaction tests</x:v>
+        <x:v>Logging redaction service and metadata audit baseline exist.</x:v>
       </x:c>
       <x:c r="L24" s="6" t="str">
         <x:v>wiki/database/data-model.md; wiki/tdd/tdd.md</x:v>
       </x:c>
-      <x:c r="M24" s="6"/>
+      <x:c r="M24" s="6" t="str">
+        <x:v>Production logging policy enforcement and durable audit persistence remain.</x:v>
+      </x:c>
       <x:c r="N24" s="6" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3366,20 +3382,20 @@
         <x:v>GET monthly monitoring endpoints return read-only month-level monitoring data with related income and expense category context; mutation endpoints are absent or forbidden</x:v>
       </x:c>
       <x:c r="I25" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="J25" s="6"/>
       <x:c r="K25" s="6" t="str">
-        <x:v>API integration and contract test results</x:v>
+        <x:v>Backend verification passed on 2026-07-04: npm --prefix service run typecheck; npm --prefix service run test; npm --prefix service run build. Monthly Monitoring read-only endpoints return app-calculated month-level monitoring data.</x:v>
       </x:c>
       <x:c r="L25" s="6" t="str">
         <x:v>wiki/api/api-specification.md; wiki/database/data-model.md</x:v>
       </x:c>
       <x:c r="M25" s="6" t="str">
-        <x:v>Do not expose edit paths for Monthly Monitoring normal app flows</x:v>
+        <x:v>No normal app mutation endpoint is exposed for Monthly Monitoring.</x:v>
       </x:c>
       <x:c r="N25" s="6" t="str">
-        <x:v>2026-07-03</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
lots of changes in front & back, almost working with some major issues version
</commit_message>
<xml_diff>
--- a/wiki/development-plan/notion-finance-development-plan.xlsx
+++ b/wiki/development-plan/notion-finance-development-plan.xlsx
@@ -6974,7 +6974,7 @@
       </c>
       <c r="D5" s="59" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" s="56" t="inlineStr">
@@ -6984,7 +6984,7 @@
       </c>
       <c r="F5" s="57" t="inlineStr">
         <is>
-          <t>Port 3001 held by orphan node PID 76992; kill needed before backend can bootstrap</t>
+          <t>Applied 001-initial-schema.sql + 002-users-schema.sql against Neon on 2026-07-09 via direct pg client; pgcrypto enabled.</t>
         </is>
       </c>
     </row>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="D6" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" s="56" t="inlineStr">
@@ -7016,7 +7016,7 @@
       </c>
       <c r="F6" s="57" t="inlineStr">
         <is>
-          <t>Verify via Neon SQL editor after A4</t>
+          <t>Verified users + user_notion_configs tables, all columns, indexes (idx_users_email, idx_user_notion_configs_user_id, uniques), and pgcrypto extension via information_schema query.</t>
         </is>
       </c>
     </row>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="D7" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="56" t="inlineStr">
@@ -7048,7 +7048,7 @@
       </c>
       <c r="F7" s="57" t="inlineStr">
         <is>
-          <t>Destructive test space per project rule</t>
+          <t>User confirmed sandbox workspace duplicated on 2026-07-09.</t>
         </is>
       </c>
     </row>
@@ -7070,7 +7070,7 @@
       </c>
       <c r="D8" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="56" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="F8" s="57" t="inlineStr">
         <is>
-          <t>Accounts, IncomeCategories, Incomes, ExpenseCategories, Expenses</t>
+          <t>Token + 6 DB IDs (accounts, incomeCategories, incomes, expenseCategories, expenses, monthlyMonitoring) received 2026-07-09 and wired into service/.env as dev fallback. Runtime path is per-user via PUT /user/notion-config.</t>
         </is>
       </c>
     </row>
@@ -7102,7 +7102,7 @@
       </c>
       <c r="D9" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E9" s="56" t="inlineStr">
@@ -7112,7 +7112,7 @@
       </c>
       <c r="F9" s="57" t="inlineStr">
         <is>
-          <t>Confirms encryption round-trip in user_notion_configs</t>
+          <t>Smoke test 2026-07-09 passed: POST /auth/register + /auth/login returned JWT; PUT /user/notion-config persisted AES-256-GCM ciphertext (iv:authTag:cipher, 3 segments) + db_ids jsonb; GET returned tokenConfigured=true confirming server-side decryption round-trip.</t>
         </is>
       </c>
     </row>
@@ -7134,7 +7134,7 @@
       </c>
       <c r="D10" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E10" s="56" t="inlineStr">
@@ -7144,7 +7144,7 @@
       </c>
       <c r="F10" s="57" t="inlineStr">
         <is>
-          <t>Per-user path decided over env token</t>
+          <t>Built app/notion-connect/page.tsx: authenticated form with token + 5 required + 1 optional DB IDs; wires userNotionConfigApi.get/save/remove; prefills dbIds from live config on mount; masks configured token; disconnect action. Typechecks; SSR renders 200 with Loading state, page shell logs no errors.</t>
         </is>
       </c>
     </row>
@@ -7166,7 +7166,7 @@
       </c>
       <c r="D11" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E11" s="56" t="inlineStr">
@@ -7174,7 +7174,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F11" s="57" t="inlineStr"/>
+      <c r="F11" s="57" t="inlineStr">
+        <is>
+          <t>GET /system/schema-status → {status:configured, missing:[], 12 checks all live} for both anon and authed calls with per-user config. Note: schemaStatus only verifies client construction, not live property/select drift — B3 handles that.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="56" t="inlineStr">
@@ -7194,7 +7198,7 @@
       </c>
       <c r="D12" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E12" s="56" t="inlineStr">
@@ -7204,7 +7208,7 @@
       </c>
       <c r="F12" s="57" t="inlineStr">
         <is>
-          <t>Depends on live schema</t>
+          <t>Live schema audit vs notion-property-mapper.ts: 0 drift. All property names + types match across accounts (12), incomeCategories (5), incomes (8), expenseCategories (8), expenses (17). All select-option unions (AccountType, PaymentStatus, PaymentFrequency, PasabuyStatus, Auxiliary Yes/No) match live options exactly. monthlyMonitoring is synthetic — not from Notion.</t>
         </is>
       </c>
     </row>
@@ -7226,7 +7230,7 @@
       </c>
       <c r="D13" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E13" s="56" t="inlineStr">
@@ -7234,7 +7238,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F13" s="57" t="inlineStr"/>
+      <c r="F13" s="57" t="inlineStr">
+        <is>
+          <t>GET list + detail return live Notion pages. Counts: accounts=15, incomeCategories=18, incomes=917, expenseCategories=37, expenses=2938. Canonical Notion page-IDs (32-hex-dash). Verified sample: account "Maya Landers (Visa)" (Credit, limit 97000, points 128.1); income "[260705] Transfer" 2026-07-05. Detail endpoint returns matching record.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="56" t="inlineStr">
@@ -7254,7 +7262,7 @@
       </c>
       <c r="D14" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E14" s="56" t="inlineStr">
@@ -7262,7 +7270,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F14" s="57" t="inlineStr"/>
+      <c r="F14" s="57" t="inlineStr">
+        <is>
+          <t>POST /incomes returned Notion page id 39847796-…-eaa6649ec646; independent Notion retrieve confirmed title, date=2026-07-09, grossIncome=123.45, Accounts + Categories relations set correctly.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="56" t="inlineStr">
@@ -7282,7 +7294,7 @@
       </c>
       <c r="D15" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E15" s="56" t="inlineStr">
@@ -7290,7 +7302,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F15" s="57" t="inlineStr"/>
+      <c r="F15" s="57" t="inlineStr">
+        <is>
+          <t>POST /expenses (base + CC link + Pasabuy fields) created page 39847796-…-ef20bf4d99b2. PATCH partial payload updated amount/paymentStatus/datePaid/pasabuyStatus/pasabuyPaidPeriod cleanly. FIX: incomeDtoToProperties + expenseDtoToProperties were emitting required fields even when omitted, converting undefined into "null" date strings, empty titles, cleared relations — refactored both builders to emit only keys present in dto; buildNotionProperties in notion.service.ts updated to match. Note: Notion silently rejects CC Link Payment Receipt relation from non-CC-payment expense targets — Notion-side schema constraint, not a mapper issue.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="56" t="inlineStr">
@@ -7310,7 +7326,7 @@
       </c>
       <c r="D16" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E16" s="56" t="inlineStr">
@@ -7320,7 +7336,7 @@
       </c>
       <c r="F16" s="57" t="inlineStr">
         <is>
-          <t>Income + Expense</t>
+          <t>DELETE /incomes/:id → Notion title "C1 E2E test 1783606267 [Deleted: 123.45]" + grossIncome=0. DELETE /expenses/:id → title "C2 E2E test 1783606267 [Deleted: 750]" + amount=0. Both pages remain non-archived; all other fields preserved (soft-delete). Mapper fix above enables this — pre-fix, delete would have clobbered untouched fields.</t>
         </is>
       </c>
     </row>
@@ -7342,7 +7358,7 @@
       </c>
       <c r="D17" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E17" s="56" t="inlineStr">
@@ -7350,7 +7366,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F17" s="57" t="inlineStr"/>
+      <c r="F17" s="57" t="inlineStr">
+        <is>
+          <t>POST /sync/commit tested twice: (1) batch of 2 creates → 2 applied/0 failed, freshSnapshot for 2026-07 contained new records (12 incomes/39 expenses in-month vs 917/2938 all-months). (2) batch of update + 2 deletes → 3 applied/0 failed, snapshot reflected [Deleted: amount] titles and zeroed values. returnFreshSnapshot + snapshotMonth both respected.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="56" t="inlineStr">
@@ -7370,7 +7390,7 @@
       </c>
       <c r="D18" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E18" s="56" t="inlineStr">
@@ -7378,7 +7398,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F18" s="57" t="inlineStr"/>
+      <c r="F18" s="57" t="inlineStr">
+        <is>
+          <t>JWT verified: exp-iat = 604800s = 7 days exactly; payload = {id,email,roles:["user"]}. /auth/logout stateless: returns {loggedOut:true}, token remains valid server-side (client discards via localStorage.removeItem in application/src/lib/auth-context.tsx:86). Fixed drift in auth.module.ts:18 so JWT_EXPIRES_IN env is now honored (was hardcoded to "7d").</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="56" t="inlineStr">
@@ -7398,7 +7422,7 @@
       </c>
       <c r="D19" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E19" s="56" t="inlineStr">
@@ -7406,7 +7430,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F19" s="57" t="inlineStr"/>
+      <c r="F19" s="57" t="inlineStr">
+        <is>
+          <t>Installed @nestjs/throttler@6.5.0. Global ThrottlerModule (100/min per IP) via APP_GUARD in app.module.ts, plus @Throttle({limit:10, ttl:60_000}) on POST /auth/login and /auth/register in auth.controller.ts. Verified: 12 rapid attempts → first 10 pass (401/201 per credentials), attempts 11-12 → 429; window resets after ttl.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="56" t="inlineStr">
@@ -7436,7 +7464,7 @@
       </c>
       <c r="F20" s="57" t="inlineStr">
         <is>
-          <t>Explicitly deferred this phase</t>
+          <t>Explicitly deferred this phase. NOTION: Google Sign-In hooks still exist in code path (auth-controller.ts imports google-auth-library, config exposes GOOGLE_CLIENT_ID/SECRET) but env is intentionally unset; server logs a boot-time warning.</t>
         </is>
       </c>
     </row>
@@ -7458,7 +7486,7 @@
       </c>
       <c r="D21" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E21" s="56" t="inlineStr">
@@ -7466,7 +7494,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F21" s="57" t="inlineStr"/>
+      <c r="F21" s="57" t="inlineStr">
+        <is>
+          <t>Replaced module-level empty Account[]/IncomeCategory[] arrays with a shared useLiveCollections() hook wired to useAccounts(true), useIncomeCategories, useExpenseCategories. IncomePage/ExpensePage now accept selectedMonth and call useIncomes/useExpenses with month + filter params; MonthlyMonitoringPage derives monitoring totals from live records; DashboardPage/WorkflowPage read active credit accounts + normal income categories from the hook. getIncomeCategorySummaries signature updated to take (records, categories). Frontend typecheck + tests green.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="56" t="inlineStr">
@@ -7486,7 +7518,7 @@
       </c>
       <c r="D22" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E22" s="56" t="inlineStr">
@@ -7494,7 +7526,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F22" s="57" t="inlineStr"/>
+      <c r="F22" s="57" t="inlineStr">
+        <is>
+          <t>Added Schema Check button to TopBar (visible from every section) wired to existing verifySchema() which calls syncApi.schemaStatus(). Sets schemaHealth pill to verified/warning based on response.success. TopBar signature gained onSchemaVerify prop.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="56" t="inlineStr">
@@ -7514,7 +7550,7 @@
       </c>
       <c r="D23" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E23" s="56" t="inlineStr">
@@ -7522,7 +7558,11 @@
           <t>Claude</t>
         </is>
       </c>
-      <c r="F23" s="57" t="inlineStr"/>
+      <c r="F23" s="57" t="inlineStr">
+        <is>
+          <t>runSync now explicitly calls syncApi.pullLatest first (accounts, incomeCategories, expenseCategories, incomes, expenses; month=selectedMonth) then syncApi.commit with operations=[], returnFreshSnapshot=true, snapshotMonth=selectedMonth. Updates lastSync + zeros pendingOperations on success. Dropped legacy setTimeout mock fallback.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="56" t="inlineStr">
@@ -7626,7 +7666,7 @@
       </c>
       <c r="D27" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E27" s="56" t="inlineStr">
@@ -7636,7 +7676,7 @@
       </c>
       <c r="F27" s="57" t="inlineStr">
         <is>
-          <t>Blocked until A-C done</t>
+          <t>Playwright 1.61.1 installed with chromium. application/playwright.config.ts boots the Next dev server on E2E_PORT=3100 with NEXT_PUBLIC_BACKEND_URL=E2E_BACKEND_URL (default :3001). e2e/auth-connect-income-sync.spec.ts: fresh-user register → /notion-connect save (token + 5 required + 1 optional DB IDs) → API cross-check config + accounts + income-categories → API create income → click TopBar Sync button → assert POST /sync/pull is issued and "Syncing" pill renders → API soft-delete for cleanup. Run: 1 passed (1.3m).</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7698,7 @@
       </c>
       <c r="D28" s="60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E28" s="56" t="inlineStr">
@@ -7668,7 +7708,7 @@
       </c>
       <c r="F28" s="57" t="inlineStr">
         <is>
-          <t>Blocked until A-C done</t>
+          <t>service/src/notion/notion.integration.spec.ts composes real @notionhq/client + NotionApiClient + property mapper against live sandbox DBs. Guards on env: skipped with a console warn when NOTION_TOKEN or the 5 DB IDs are absent, so CI without secrets stays green. Covers create → partial update (proves C2 mapper fix on server-side too) → soft-delete round-trip for both Incomes and Expenses. Suite: 2 passed (30s). Backend total: 4 files / 12 tests passing.</t>
         </is>
       </c>
     </row>

</xml_diff>